<commit_message>
before to go payroll screen
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="67">
   <si>
     <t/>
   </si>
@@ -212,6 +212,9 @@
   </si>
   <si>
     <t>22/06/2026 01:10 م</t>
+  </si>
+  <si>
+    <t>nor ahmed</t>
   </si>
 </sst>
 </file>
@@ -1867,114 +1870,290 @@
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="1"/>
-      <c r="B51" s="1"/>
-      <c r="C51" s="1"/>
-      <c r="D51" s="1"/>
-      <c r="E51" s="1"/>
-      <c r="F51" s="1"/>
-      <c r="G51" s="1"/>
-      <c r="H51" s="1"/>
+      <c r="A51" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="1"/>
-      <c r="B52" s="1"/>
-      <c r="C52" s="1"/>
-      <c r="D52" s="1"/>
-      <c r="E52" s="1"/>
-      <c r="F52" s="1"/>
-      <c r="G52" s="1"/>
-      <c r="H52" s="1"/>
+      <c r="A52" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="1"/>
-      <c r="B53" s="1"/>
-      <c r="C53" s="1"/>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1"/>
-      <c r="G53" s="1"/>
-      <c r="H53" s="1"/>
+      <c r="A53" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="1"/>
-      <c r="B54" s="1"/>
-      <c r="C54" s="1"/>
-      <c r="D54" s="1"/>
-      <c r="E54" s="1"/>
-      <c r="F54" s="1"/>
-      <c r="G54" s="1"/>
-      <c r="H54" s="1"/>
+      <c r="A54" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="1"/>
-      <c r="D55" s="1"/>
-      <c r="E55" s="1"/>
-      <c r="F55" s="1"/>
-      <c r="G55" s="1"/>
-      <c r="H55" s="1"/>
+      <c r="A55" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="1"/>
-      <c r="B56" s="1"/>
-      <c r="C56" s="1"/>
-      <c r="D56" s="1"/>
-      <c r="E56" s="1"/>
-      <c r="F56" s="1"/>
-      <c r="G56" s="1"/>
-      <c r="H56" s="1"/>
+      <c r="A56" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C56" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G56" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="1"/>
-      <c r="B57" s="1"/>
-      <c r="C57" s="1"/>
-      <c r="D57" s="1"/>
-      <c r="E57" s="1"/>
-      <c r="F57" s="1"/>
-      <c r="G57" s="1"/>
-      <c r="H57" s="1"/>
+      <c r="A57" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C57" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="1"/>
-      <c r="B58" s="1"/>
-      <c r="C58" s="1"/>
-      <c r="D58" s="1"/>
-      <c r="E58" s="1"/>
-      <c r="F58" s="1"/>
-      <c r="G58" s="1"/>
-      <c r="H58" s="1"/>
+      <c r="A58" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C58" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="1"/>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
-      <c r="H59" s="1"/>
+      <c r="A59" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C59" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="1"/>
-      <c r="B60" s="1"/>
-      <c r="C60" s="1"/>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1"/>
-      <c r="G60" s="1"/>
-      <c r="H60" s="1"/>
+      <c r="A60" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C60" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="1"/>
-      <c r="B61" s="1"/>
-      <c r="C61" s="1"/>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1"/>
-      <c r="G61" s="1"/>
-      <c r="H61" s="1"/>
+      <c r="A61" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G61" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>

</xml_diff>

<commit_message>
still some fixes before screen 2
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="67">
   <si>
     <t/>
   </si>
@@ -562,7 +562,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H301"/>
+  <dimension ref="A1:H292"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1922,238 +1922,94 @@
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C53" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H53" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A53" s="1"/>
+      <c r="B53" s="1"/>
+      <c r="C53" s="1"/>
+      <c r="D53" s="1"/>
+      <c r="E53" s="1"/>
+      <c r="F53" s="1"/>
+      <c r="G53" s="1"/>
+      <c r="H53" s="1"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D54" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="E54" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F54" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G54" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H54" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A54" s="1"/>
+      <c r="B54" s="1"/>
+      <c r="C54" s="1"/>
+      <c r="D54" s="1"/>
+      <c r="E54" s="1"/>
+      <c r="F54" s="1"/>
+      <c r="G54" s="1"/>
+      <c r="H54" s="1"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B55" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C55" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F55" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A55" s="1"/>
+      <c r="B55" s="1"/>
+      <c r="C55" s="1"/>
+      <c r="D55" s="1"/>
+      <c r="E55" s="1"/>
+      <c r="F55" s="1"/>
+      <c r="G55" s="1"/>
+      <c r="H55" s="1"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C56" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F56" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A56" s="1"/>
+      <c r="B56" s="1"/>
+      <c r="C56" s="1"/>
+      <c r="D56" s="1"/>
+      <c r="E56" s="1"/>
+      <c r="F56" s="1"/>
+      <c r="G56" s="1"/>
+      <c r="H56" s="1"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A57" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B57" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A57" s="1"/>
+      <c r="B57" s="1"/>
+      <c r="C57" s="1"/>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
+      <c r="F57" s="1"/>
+      <c r="G57" s="1"/>
+      <c r="H57" s="1"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B58" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F58" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A58" s="1"/>
+      <c r="B58" s="1"/>
+      <c r="C58" s="1"/>
+      <c r="D58" s="1"/>
+      <c r="E58" s="1"/>
+      <c r="F58" s="1"/>
+      <c r="G58" s="1"/>
+      <c r="H58" s="1"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B59" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C59" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F59" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A59" s="1"/>
+      <c r="B59" s="1"/>
+      <c r="C59" s="1"/>
+      <c r="D59" s="1"/>
+      <c r="E59" s="1"/>
+      <c r="F59" s="1"/>
+      <c r="G59" s="1"/>
+      <c r="H59" s="1"/>
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A60" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B60" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F60" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H60" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A60" s="1"/>
+      <c r="B60" s="1"/>
+      <c r="C60" s="1"/>
+      <c r="D60" s="1"/>
+      <c r="E60" s="1"/>
+      <c r="F60" s="1"/>
+      <c r="G60" s="1"/>
+      <c r="H60" s="1"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C61" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F61" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>0</v>
-      </c>
+      <c r="A61" s="1"/>
+      <c r="B61" s="1"/>
+      <c r="C61" s="1"/>
+      <c r="D61" s="1"/>
+      <c r="E61" s="1"/>
+      <c r="F61" s="1"/>
+      <c r="G61" s="1"/>
+      <c r="H61" s="1"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62" s="1"/>
@@ -4261,7 +4117,7 @@
       <c r="C272" s="1"/>
       <c r="D272" s="1"/>
       <c r="E272" s="1"/>
-      <c r="F272" s="1"/>
+      <c r="F272" s="3"/>
       <c r="G272" s="1"/>
       <c r="H272" s="1"/>
     </row>
@@ -4271,7 +4127,7 @@
       <c r="C273" s="1"/>
       <c r="D273" s="1"/>
       <c r="E273" s="1"/>
-      <c r="F273" s="1"/>
+      <c r="F273" s="3"/>
       <c r="G273" s="1"/>
       <c r="H273" s="1"/>
     </row>
@@ -4311,7 +4167,7 @@
       <c r="C277" s="1"/>
       <c r="D277" s="1"/>
       <c r="E277" s="1"/>
-      <c r="F277" s="1"/>
+      <c r="F277" s="3"/>
       <c r="G277" s="1"/>
       <c r="H277" s="1"/>
     </row>
@@ -4351,7 +4207,7 @@
       <c r="C281" s="1"/>
       <c r="D281" s="1"/>
       <c r="E281" s="1"/>
-      <c r="F281" s="3"/>
+      <c r="F281" s="1"/>
       <c r="G281" s="1"/>
       <c r="H281" s="1"/>
     </row>
@@ -4361,7 +4217,7 @@
       <c r="C282" s="1"/>
       <c r="D282" s="1"/>
       <c r="E282" s="1"/>
-      <c r="F282" s="3"/>
+      <c r="F282" s="1"/>
       <c r="G282" s="1"/>
       <c r="H282" s="1"/>
     </row>
@@ -4401,7 +4257,7 @@
       <c r="C286" s="1"/>
       <c r="D286" s="1"/>
       <c r="E286" s="1"/>
-      <c r="F286" s="3"/>
+      <c r="F286" s="1"/>
       <c r="G286" s="1"/>
       <c r="H286" s="1"/>
     </row>
@@ -4465,96 +4321,6 @@
       <c r="G292" s="1"/>
       <c r="H292" s="1"/>
     </row>
-    <row r="293" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A293" s="1"/>
-      <c r="B293" s="1"/>
-      <c r="C293" s="1"/>
-      <c r="D293" s="1"/>
-      <c r="E293" s="1"/>
-      <c r="F293" s="1"/>
-      <c r="G293" s="1"/>
-      <c r="H293" s="1"/>
-    </row>
-    <row r="294" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A294" s="1"/>
-      <c r="B294" s="1"/>
-      <c r="C294" s="1"/>
-      <c r="D294" s="1"/>
-      <c r="E294" s="1"/>
-      <c r="F294" s="1"/>
-      <c r="G294" s="1"/>
-      <c r="H294" s="1"/>
-    </row>
-    <row r="295" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A295" s="1"/>
-      <c r="B295" s="1"/>
-      <c r="C295" s="1"/>
-      <c r="D295" s="1"/>
-      <c r="E295" s="1"/>
-      <c r="F295" s="1"/>
-      <c r="G295" s="1"/>
-      <c r="H295" s="1"/>
-    </row>
-    <row r="296" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A296" s="1"/>
-      <c r="B296" s="1"/>
-      <c r="C296" s="1"/>
-      <c r="D296" s="1"/>
-      <c r="E296" s="1"/>
-      <c r="F296" s="1"/>
-      <c r="G296" s="1"/>
-      <c r="H296" s="1"/>
-    </row>
-    <row r="297" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A297" s="1"/>
-      <c r="B297" s="1"/>
-      <c r="C297" s="1"/>
-      <c r="D297" s="1"/>
-      <c r="E297" s="1"/>
-      <c r="F297" s="1"/>
-      <c r="G297" s="1"/>
-      <c r="H297" s="1"/>
-    </row>
-    <row r="298" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A298" s="1"/>
-      <c r="B298" s="1"/>
-      <c r="C298" s="1"/>
-      <c r="D298" s="1"/>
-      <c r="E298" s="1"/>
-      <c r="F298" s="1"/>
-      <c r="G298" s="1"/>
-      <c r="H298" s="1"/>
-    </row>
-    <row r="299" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A299" s="1"/>
-      <c r="B299" s="1"/>
-      <c r="C299" s="1"/>
-      <c r="D299" s="1"/>
-      <c r="E299" s="1"/>
-      <c r="F299" s="1"/>
-      <c r="G299" s="1"/>
-      <c r="H299" s="1"/>
-    </row>
-    <row r="300" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A300" s="1"/>
-      <c r="B300" s="1"/>
-      <c r="C300" s="1"/>
-      <c r="D300" s="1"/>
-      <c r="E300" s="1"/>
-      <c r="F300" s="1"/>
-      <c r="G300" s="1"/>
-      <c r="H300" s="1"/>
-    </row>
-    <row r="301" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A301" s="1"/>
-      <c r="B301" s="1"/>
-      <c r="C301" s="1"/>
-      <c r="D301" s="1"/>
-      <c r="E301" s="1"/>
-      <c r="F301" s="1"/>
-      <c r="G301" s="1"/>
-      <c r="H301" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter>

</xml_diff>